<commit_message>
Atualização planilha de exemplo
</commit_message>
<xml_diff>
--- a/ExcelDoc/ExcelDoc.Server/Planilha/Planilha Exemplo.xlsx
+++ b/ExcelDoc/ExcelDoc.Server/Planilha/Planilha Exemplo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilso\OneDrive\Área de Trabalho\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B09E24E-BF7D-4B6F-8A86-7BF1CD297E90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE58501-540F-4186-B99E-25032CB04967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="842" xr2:uid="{2FB819D7-AF95-4E9E-9F21-A2B99D445FA7}"/>
   </bookViews>
@@ -567,7 +567,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -631,14 +631,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -688,48 +698,64 @@
     <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{018748D7-2EEA-4364-97F9-8DEB3207DD3F}"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <color rgb="FFB91C1C"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FFB91C1C"/>
@@ -801,8 +827,8 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Estilo de Tabela 1" pivot="0" count="2" xr9:uid="{68D78791-29AF-48EF-A089-07006C6F704C}">
-      <tableStyleElement type="wholeTable" dxfId="3"/>
-      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="wholeTable" dxfId="4"/>
+      <tableStyleElement type="headerRow" dxfId="3"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -814,10 +840,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1120,306 +1142,307 @@
   <dimension ref="A1:AM22"/>
   <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" customWidth="1"/>
-    <col min="9" max="9" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.140625" customWidth="1"/>
-    <col min="11" max="11" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.7109375" customWidth="1"/>
-    <col min="17" max="17" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="19.42578125" customWidth="1"/>
-    <col min="20" max="24" width="34" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="58.85546875" customWidth="1"/>
-    <col min="31" max="31" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="32.85546875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="28.5703125" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="25" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="33" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="52" customWidth="1"/>
+    <col min="1" max="1" width="5" style="27" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" style="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24" style="27" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.140625" style="27" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.140625" style="27" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.5703125" style="27" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.7109375" style="27" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" style="27" customWidth="1"/>
+    <col min="9" max="9" width="29.42578125" style="27" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.140625" style="27" customWidth="1"/>
+    <col min="11" max="11" width="18.5703125" style="27" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.42578125" style="27" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.7109375" style="27" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.7109375" style="27" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.28515625" style="27" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.7109375" style="27" customWidth="1"/>
+    <col min="17" max="17" width="23.5703125" style="27" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="26.140625" style="27" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.42578125" style="27" customWidth="1"/>
+    <col min="20" max="24" width="34" style="27" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="22.7109375" style="27" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="25.28515625" style="31" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="22.42578125" style="27" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="22.28515625" style="27" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="16.140625" style="27" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="58.85546875" style="27" customWidth="1"/>
+    <col min="31" max="31" width="20.28515625" style="27" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="27.140625" style="27" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="27.28515625" style="27" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="32.85546875" style="27" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.5703125" style="27" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="28.5703125" style="27" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="25" style="27" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="33" style="27" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="52" style="27" customWidth="1"/>
+    <col min="40" max="16384" width="9.140625" style="27"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" s="2" customFormat="1" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:39" s="1" customFormat="1" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="O1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="Q1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="R1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="S1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="T1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="U1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="V1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="W1" s="5" t="s">
+      <c r="W1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="X1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="Y1" s="5" t="s">
+      <c r="Y1" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="Z1" s="5" t="s">
+      <c r="Z1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="AA1" s="5" t="s">
+      <c r="AA1" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="AB1" s="5" t="s">
+      <c r="AB1" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="AC1" s="6" t="s">
+      <c r="AC1" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="AD1" s="6" t="s">
+      <c r="AD1" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="AE1" s="7" t="s">
+      <c r="AE1" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="AF1" s="7" t="s">
+      <c r="AF1" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="AG1" s="8" t="s">
+      <c r="AG1" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="AH1" s="8" t="s">
+      <c r="AH1" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="AI1" s="8" t="s">
+      <c r="AI1" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="AJ1" s="8" t="s">
+      <c r="AJ1" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="AK1" s="8" t="s">
+      <c r="AK1" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="AL1" s="8" t="s">
+      <c r="AL1" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="AM1" s="8" t="s">
+      <c r="AM1" s="7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:39" s="3" customFormat="1" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
+    <row r="2" spans="1:39" s="2" customFormat="1" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="J2" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="K2" s="10" t="s">
+      <c r="K2" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="L2" s="10" t="s">
+      <c r="L2" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="M2" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="N2" s="11" t="s">
+      <c r="N2" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="P2" s="12" t="s">
+      <c r="P2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="Q2" s="13" t="s">
+      <c r="Q2" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="R2" s="13" t="s">
+      <c r="R2" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="S2" s="13" t="s">
+      <c r="S2" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="T2" s="13" t="s">
+      <c r="T2" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="U2" s="13" t="s">
+      <c r="U2" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="V2" s="13" t="s">
+      <c r="V2" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W2" s="13" t="s">
+      <c r="W2" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="X2" s="13" t="s">
+      <c r="X2" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="Y2" s="13" t="s">
+      <c r="Y2" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="Z2" s="13" t="s">
+      <c r="Z2" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="AA2" s="13" t="s">
+      <c r="AA2" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="AB2" s="13" t="s">
+      <c r="AB2" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="AC2" s="14" t="s">
+      <c r="AC2" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="AD2" s="14" t="s">
+      <c r="AD2" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="AE2" s="15" t="s">
+      <c r="AE2" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="AF2" s="15" t="s">
+      <c r="AF2" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="AG2" s="15" t="s">
+      <c r="AG2" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="AH2" s="15" t="s">
+      <c r="AH2" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="AI2" s="15" t="s">
+      <c r="AI2" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="AJ2" s="15" t="s">
+      <c r="AJ2" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="AK2" s="15" t="s">
+      <c r="AK2" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="AL2" s="15" t="s">
+      <c r="AL2" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="AM2" s="16" t="s">
+      <c r="AM2" s="15" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="A3" s="27">
         <v>1</v>
       </c>
-      <c r="B3" s="19">
+      <c r="B3" s="23">
         <v>46231</v>
       </c>
-      <c r="C3" s="19">
+      <c r="C3" s="23">
         <v>46231</v>
       </c>
-      <c r="D3" s="19">
+      <c r="D3" s="23">
         <v>46231</v>
       </c>
-      <c r="E3" s="20">
+      <c r="E3" s="28">
         <v>1</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="F3" s="22" t="s">
         <v>77</v>
       </c>
       <c r="G3" s="22"/>
       <c r="H3" s="22"/>
-      <c r="I3" s="23">
+      <c r="I3" s="24">
         <v>-1</v>
       </c>
-      <c r="J3" s="24">
+      <c r="J3" s="18">
         <v>100001</v>
       </c>
       <c r="K3" s="22"/>
@@ -1430,13 +1453,13 @@
       <c r="N3" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="O3" s="25">
+      <c r="O3" s="19">
         <v>1</v>
       </c>
-      <c r="P3" s="25">
+      <c r="P3" s="19">
         <v>10000</v>
       </c>
-      <c r="Q3" s="23">
+      <c r="Q3" s="24">
         <v>22</v>
       </c>
       <c r="R3" s="22" t="s">
@@ -1453,14 +1476,14 @@
       <c r="Y3" s="22">
         <v>1101001001</v>
       </c>
-      <c r="Z3" s="22"/>
+      <c r="Z3" s="29"/>
       <c r="AA3" s="22"/>
       <c r="AB3" s="22">
         <v>0</v>
       </c>
       <c r="AC3" s="22"/>
       <c r="AD3" s="22"/>
-      <c r="AE3" s="26"/>
+      <c r="AE3" s="25"/>
       <c r="AF3" s="22"/>
       <c r="AG3" s="22"/>
       <c r="AH3" s="22"/>
@@ -1471,31 +1494,31 @@
       <c r="AM3" s="22"/>
     </row>
     <row r="4" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="A4" s="27">
         <v>2</v>
       </c>
-      <c r="B4" s="19">
+      <c r="B4" s="23">
         <v>46113</v>
       </c>
-      <c r="C4" s="27">
+      <c r="C4" s="23">
         <v>46104</v>
       </c>
-      <c r="D4" s="27">
+      <c r="D4" s="23">
         <v>46122</v>
       </c>
       <c r="E4" s="28">
         <v>1</v>
       </c>
-      <c r="F4" s="21" t="s">
+      <c r="F4" s="22" t="s">
         <v>77</v>
       </c>
       <c r="G4" s="22"/>
       <c r="H4" s="22"/>
-      <c r="I4" s="23">
+      <c r="I4" s="24">
         <v>-1</v>
       </c>
-      <c r="J4" s="29">
-        <v>300003</v>
+      <c r="J4" s="20">
+        <v>400004</v>
       </c>
       <c r="K4" s="22"/>
       <c r="L4" s="22"/>
@@ -1505,13 +1528,13 @@
       <c r="N4" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="O4" s="25">
+      <c r="O4" s="19">
         <v>1</v>
       </c>
-      <c r="P4" s="30">
+      <c r="P4" s="21">
         <v>50000</v>
       </c>
-      <c r="Q4" s="23">
+      <c r="Q4" s="24">
         <v>22</v>
       </c>
       <c r="R4" s="22" t="s">
@@ -1528,14 +1551,14 @@
       <c r="Y4" s="22">
         <v>1101001001</v>
       </c>
-      <c r="Z4" s="22"/>
+      <c r="Z4" s="29"/>
       <c r="AA4" s="22"/>
       <c r="AB4" s="22">
         <v>0</v>
       </c>
       <c r="AC4" s="22"/>
       <c r="AD4" s="22"/>
-      <c r="AE4" s="26"/>
+      <c r="AE4" s="25"/>
       <c r="AF4" s="22"/>
       <c r="AG4" s="22"/>
       <c r="AH4" s="22"/>
@@ -1545,27 +1568,552 @@
       <c r="AL4" s="22"/>
       <c r="AM4" s="22"/>
     </row>
-    <row r="22" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H22" s="1"/>
+    <row r="5" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="B5" s="23"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="21"/>
+      <c r="Q5" s="24"/>
+      <c r="R5" s="22"/>
+      <c r="S5" s="22"/>
+      <c r="T5" s="22"/>
+      <c r="U5" s="22"/>
+      <c r="V5" s="22"/>
+      <c r="W5" s="22"/>
+      <c r="X5" s="22"/>
+      <c r="Y5" s="22"/>
+      <c r="Z5" s="29"/>
+      <c r="AA5" s="22"/>
+      <c r="AB5" s="22"/>
+      <c r="AC5" s="22"/>
+      <c r="AD5" s="22"/>
+      <c r="AE5" s="25"/>
+      <c r="AF5" s="22"/>
+      <c r="AG5" s="22"/>
+      <c r="AH5" s="22"/>
+      <c r="AI5" s="22"/>
+      <c r="AJ5" s="22"/>
+      <c r="AK5" s="22"/>
+      <c r="AL5" s="22"/>
+      <c r="AM5" s="22"/>
+    </row>
+    <row r="6" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="19"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="24"/>
+      <c r="R6" s="22"/>
+      <c r="S6" s="22"/>
+      <c r="T6" s="22"/>
+      <c r="U6" s="22"/>
+      <c r="V6" s="22"/>
+      <c r="W6" s="22"/>
+      <c r="X6" s="22"/>
+      <c r="Y6" s="22"/>
+      <c r="Z6" s="29"/>
+      <c r="AA6" s="22"/>
+      <c r="AB6" s="22"/>
+      <c r="AC6" s="22"/>
+      <c r="AD6" s="22"/>
+      <c r="AE6" s="25"/>
+      <c r="AF6" s="22"/>
+      <c r="AG6" s="22"/>
+      <c r="AH6" s="22"/>
+      <c r="AI6" s="22"/>
+      <c r="AJ6" s="22"/>
+      <c r="AK6" s="22"/>
+      <c r="AL6" s="22"/>
+      <c r="AM6" s="22"/>
+    </row>
+    <row r="7" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="20"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="21"/>
+      <c r="Q7" s="24"/>
+      <c r="R7" s="22"/>
+      <c r="S7" s="22"/>
+      <c r="T7" s="22"/>
+      <c r="U7" s="22"/>
+      <c r="V7" s="22"/>
+      <c r="W7" s="22"/>
+      <c r="X7" s="22"/>
+      <c r="Y7" s="22"/>
+      <c r="Z7" s="29"/>
+      <c r="AA7" s="22"/>
+      <c r="AB7" s="22"/>
+      <c r="AC7" s="22"/>
+      <c r="AD7" s="22"/>
+      <c r="AE7" s="25"/>
+      <c r="AF7" s="22"/>
+      <c r="AG7" s="22"/>
+      <c r="AH7" s="22"/>
+      <c r="AI7" s="22"/>
+      <c r="AJ7" s="22"/>
+      <c r="AK7" s="22"/>
+      <c r="AL7" s="22"/>
+      <c r="AM7" s="22"/>
+    </row>
+    <row r="8" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="24"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="21"/>
+      <c r="Q8" s="24"/>
+      <c r="R8" s="22"/>
+      <c r="S8" s="22"/>
+      <c r="T8" s="22"/>
+      <c r="U8" s="22"/>
+      <c r="V8" s="22"/>
+      <c r="W8" s="22"/>
+      <c r="X8" s="22"/>
+      <c r="Y8" s="22"/>
+      <c r="Z8" s="29"/>
+      <c r="AA8" s="22"/>
+      <c r="AB8" s="22"/>
+      <c r="AC8" s="22"/>
+      <c r="AD8" s="22"/>
+      <c r="AE8" s="25"/>
+      <c r="AF8" s="22"/>
+      <c r="AG8" s="22"/>
+      <c r="AH8" s="22"/>
+      <c r="AI8" s="22"/>
+      <c r="AJ8" s="22"/>
+      <c r="AK8" s="22"/>
+      <c r="AL8" s="22"/>
+      <c r="AM8" s="22"/>
+    </row>
+    <row r="9" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="24"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="21"/>
+      <c r="Q9" s="24"/>
+      <c r="R9" s="22"/>
+      <c r="S9" s="22"/>
+      <c r="T9" s="22"/>
+      <c r="U9" s="22"/>
+      <c r="V9" s="22"/>
+      <c r="W9" s="22"/>
+      <c r="X9" s="22"/>
+      <c r="Y9" s="22"/>
+      <c r="Z9" s="29"/>
+      <c r="AA9" s="22"/>
+      <c r="AB9" s="22"/>
+      <c r="AC9" s="22"/>
+      <c r="AD9" s="22"/>
+      <c r="AE9" s="25"/>
+      <c r="AF9" s="22"/>
+      <c r="AG9" s="22"/>
+      <c r="AH9" s="22"/>
+      <c r="AI9" s="22"/>
+      <c r="AJ9" s="22"/>
+      <c r="AK9" s="22"/>
+      <c r="AL9" s="22"/>
+      <c r="AM9" s="22"/>
+    </row>
+    <row r="10" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="20"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="22"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="19"/>
+      <c r="P10" s="21"/>
+      <c r="Q10" s="24"/>
+      <c r="R10" s="22"/>
+      <c r="S10" s="22"/>
+      <c r="T10" s="22"/>
+      <c r="U10" s="22"/>
+      <c r="V10" s="22"/>
+      <c r="W10" s="22"/>
+      <c r="X10" s="22"/>
+      <c r="Y10" s="22"/>
+      <c r="Z10" s="29"/>
+      <c r="AA10" s="22"/>
+      <c r="AB10" s="22"/>
+      <c r="AC10" s="22"/>
+      <c r="AD10" s="22"/>
+      <c r="AE10" s="25"/>
+      <c r="AF10" s="22"/>
+      <c r="AG10" s="22"/>
+      <c r="AH10" s="22"/>
+      <c r="AI10" s="22"/>
+      <c r="AJ10" s="22"/>
+      <c r="AK10" s="22"/>
+      <c r="AL10" s="22"/>
+      <c r="AM10" s="22"/>
+    </row>
+    <row r="11" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="20"/>
+      <c r="K11" s="22"/>
+      <c r="L11" s="22"/>
+      <c r="M11" s="22"/>
+      <c r="N11" s="22"/>
+      <c r="O11" s="19"/>
+      <c r="P11" s="21"/>
+      <c r="Q11" s="24"/>
+      <c r="R11" s="22"/>
+      <c r="S11" s="22"/>
+      <c r="T11" s="22"/>
+      <c r="U11" s="22"/>
+      <c r="V11" s="22"/>
+      <c r="W11" s="22"/>
+      <c r="X11" s="22"/>
+      <c r="Y11" s="22"/>
+      <c r="Z11" s="29"/>
+      <c r="AA11" s="22"/>
+      <c r="AB11" s="22"/>
+      <c r="AC11" s="22"/>
+      <c r="AD11" s="22"/>
+      <c r="AE11" s="25"/>
+      <c r="AF11" s="22"/>
+      <c r="AG11" s="22"/>
+      <c r="AH11" s="22"/>
+      <c r="AI11" s="22"/>
+      <c r="AJ11" s="22"/>
+      <c r="AK11" s="22"/>
+      <c r="AL11" s="22"/>
+      <c r="AM11" s="22"/>
+    </row>
+    <row r="12" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="22"/>
+      <c r="L12" s="22"/>
+      <c r="M12" s="22"/>
+      <c r="N12" s="22"/>
+      <c r="O12" s="19"/>
+      <c r="P12" s="21"/>
+      <c r="Q12" s="24"/>
+      <c r="R12" s="22"/>
+      <c r="S12" s="22"/>
+      <c r="T12" s="22"/>
+      <c r="U12" s="22"/>
+      <c r="V12" s="22"/>
+      <c r="W12" s="22"/>
+      <c r="X12" s="22"/>
+      <c r="Y12" s="22"/>
+      <c r="Z12" s="29"/>
+      <c r="AA12" s="22"/>
+      <c r="AB12" s="22"/>
+      <c r="AC12" s="22"/>
+      <c r="AD12" s="22"/>
+      <c r="AE12" s="25"/>
+      <c r="AF12" s="22"/>
+      <c r="AG12" s="22"/>
+      <c r="AH12" s="22"/>
+      <c r="AI12" s="22"/>
+      <c r="AJ12" s="22"/>
+      <c r="AK12" s="22"/>
+      <c r="AL12" s="22"/>
+      <c r="AM12" s="22"/>
+    </row>
+    <row r="13" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="24"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="22"/>
+      <c r="L13" s="22"/>
+      <c r="M13" s="22"/>
+      <c r="N13" s="22"/>
+      <c r="O13" s="19"/>
+      <c r="P13" s="21"/>
+      <c r="Q13" s="24"/>
+      <c r="R13" s="22"/>
+      <c r="S13" s="22"/>
+      <c r="T13" s="22"/>
+      <c r="U13" s="22"/>
+      <c r="V13" s="22"/>
+      <c r="W13" s="22"/>
+      <c r="X13" s="22"/>
+      <c r="Y13" s="22"/>
+      <c r="Z13" s="29"/>
+      <c r="AA13" s="22"/>
+      <c r="AB13" s="22"/>
+      <c r="AC13" s="22"/>
+      <c r="AD13" s="22"/>
+      <c r="AE13" s="25"/>
+      <c r="AF13" s="22"/>
+      <c r="AG13" s="22"/>
+      <c r="AH13" s="22"/>
+      <c r="AI13" s="22"/>
+      <c r="AJ13" s="22"/>
+      <c r="AK13" s="22"/>
+      <c r="AL13" s="22"/>
+      <c r="AM13" s="22"/>
+    </row>
+    <row r="14" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="24"/>
+      <c r="J14" s="20"/>
+      <c r="K14" s="22"/>
+      <c r="L14" s="22"/>
+      <c r="M14" s="22"/>
+      <c r="N14" s="22"/>
+      <c r="O14" s="19"/>
+      <c r="P14" s="21"/>
+      <c r="Q14" s="24"/>
+      <c r="R14" s="22"/>
+      <c r="S14" s="22"/>
+      <c r="T14" s="22"/>
+      <c r="U14" s="22"/>
+      <c r="V14" s="22"/>
+      <c r="W14" s="22"/>
+      <c r="X14" s="22"/>
+      <c r="Y14" s="22"/>
+      <c r="Z14" s="29"/>
+      <c r="AA14" s="22"/>
+      <c r="AB14" s="22"/>
+      <c r="AC14" s="22"/>
+      <c r="AD14" s="22"/>
+      <c r="AE14" s="25"/>
+      <c r="AF14" s="22"/>
+      <c r="AG14" s="22"/>
+      <c r="AH14" s="22"/>
+      <c r="AI14" s="22"/>
+      <c r="AJ14" s="22"/>
+      <c r="AK14" s="22"/>
+      <c r="AL14" s="22"/>
+      <c r="AM14" s="22"/>
+    </row>
+    <row r="15" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="24"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="22"/>
+      <c r="L15" s="22"/>
+      <c r="M15" s="22"/>
+      <c r="N15" s="22"/>
+      <c r="O15" s="19"/>
+      <c r="P15" s="21"/>
+      <c r="Q15" s="24"/>
+      <c r="R15" s="22"/>
+      <c r="S15" s="22"/>
+      <c r="T15" s="22"/>
+      <c r="U15" s="22"/>
+      <c r="V15" s="22"/>
+      <c r="W15" s="22"/>
+      <c r="X15" s="22"/>
+      <c r="Y15" s="22"/>
+      <c r="Z15" s="29"/>
+      <c r="AA15" s="22"/>
+      <c r="AB15" s="22"/>
+      <c r="AC15" s="22"/>
+      <c r="AD15" s="22"/>
+      <c r="AE15" s="25"/>
+      <c r="AF15" s="22"/>
+      <c r="AG15" s="22"/>
+      <c r="AH15" s="22"/>
+      <c r="AI15" s="22"/>
+      <c r="AJ15" s="22"/>
+      <c r="AK15" s="22"/>
+      <c r="AL15" s="22"/>
+      <c r="AM15" s="22"/>
+    </row>
+    <row r="16" spans="1:39" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="24"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="22"/>
+      <c r="L16" s="22"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="19"/>
+      <c r="P16" s="21"/>
+      <c r="Q16" s="24"/>
+      <c r="R16" s="22"/>
+      <c r="S16" s="22"/>
+      <c r="T16" s="22"/>
+      <c r="U16" s="22"/>
+      <c r="V16" s="22"/>
+      <c r="W16" s="22"/>
+      <c r="X16" s="22"/>
+      <c r="Y16" s="22"/>
+      <c r="Z16" s="29"/>
+      <c r="AA16" s="22"/>
+      <c r="AB16" s="22"/>
+      <c r="AC16" s="22"/>
+      <c r="AD16" s="22"/>
+      <c r="AE16" s="25"/>
+      <c r="AF16" s="22"/>
+      <c r="AG16" s="22"/>
+      <c r="AH16" s="22"/>
+      <c r="AI16" s="22"/>
+      <c r="AJ16" s="22"/>
+      <c r="AK16" s="22"/>
+      <c r="AL16" s="22"/>
+      <c r="AM16" s="22"/>
+    </row>
+    <row r="17" spans="2:39" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
+      <c r="I17" s="24"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="19"/>
+      <c r="P17" s="21"/>
+      <c r="Q17" s="24"/>
+      <c r="R17" s="22"/>
+      <c r="S17" s="22"/>
+      <c r="T17" s="22"/>
+      <c r="U17" s="22"/>
+      <c r="V17" s="22"/>
+      <c r="W17" s="22"/>
+      <c r="X17" s="22"/>
+      <c r="Y17" s="22"/>
+      <c r="Z17" s="29"/>
+      <c r="AA17" s="22"/>
+      <c r="AB17" s="22"/>
+      <c r="AC17" s="22"/>
+      <c r="AD17" s="22"/>
+      <c r="AE17" s="25"/>
+      <c r="AF17" s="22"/>
+      <c r="AG17" s="22"/>
+      <c r="AH17" s="22"/>
+      <c r="AI17" s="22"/>
+      <c r="AJ17" s="22"/>
+      <c r="AK17" s="22"/>
+      <c r="AL17" s="22"/>
+      <c r="AM17" s="22"/>
+    </row>
+    <row r="22" spans="2:39" x14ac:dyDescent="0.25">
+      <c r="H22" s="30"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="B3:B4 E3:F4 N3:P4">
-    <cfRule type="expression" dxfId="1" priority="2">
+  <conditionalFormatting sqref="B3:B17 E3:F17 N3:P17">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>AND(COUNTA($B3:$AM3)&gt;0,B3="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C3:D3">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>AND(COUNTA($B3:$AM3)&gt;0,C3="")</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C8:D17">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>AND(COUNTA($B8:$AM8)&gt;0,C8="")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" sqref="B3:D4" xr:uid="{D0A375CC-FD5B-4CCA-83F9-EA5AD5873474}">
+    <dataValidation type="date" sqref="B3:D17" xr:uid="{D0A375CC-FD5B-4CCA-83F9-EA5AD5873474}">
       <formula1>DATE(2000,1,1)</formula1>
       <formula2>DATE(2099,12,31)</formula2>
     </dataValidation>
-    <dataValidation type="list" sqref="S3:AD4" xr:uid="{82E79D67-1CF6-4D70-B36C-F68DCC68374E}">
+    <dataValidation type="list" sqref="S3:AD17" xr:uid="{82E79D67-1CF6-4D70-B36C-F68DCC68374E}">
       <formula1>"Sim,Não,tYES,tNO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1576,18 +2124,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Flow_SignoffStatus xmlns="086b6104-a044-4b77-af40-37bf74d909c3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="223469b0-54b4-4219-b9f2-328d01909222" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="086b6104-a044-4b77-af40-37bf74d909c3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1596,7 +2132,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101002D42A22A55248D44993FE65ADB876541" ma:contentTypeVersion="14" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="1d614a93a5190796232e272b802a6279">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="086b6104-a044-4b77-af40-37bf74d909c3" xmlns:ns3="fe7c13d1-16b7-4a4a-9330-93950a409cc6" xmlns:ns4="223469b0-54b4-4219-b9f2-328d01909222" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1b125a0b543c8e561557830048a62454" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="086b6104-a044-4b77-af40-37bf74d909c3"/>
@@ -1830,18 +2366,19 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6E18965-B26D-4362-B735-99223F49F9C5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="086b6104-a044-4b77-af40-37bf74d909c3"/>
-    <ds:schemaRef ds:uri="223469b0-54b4-4219-b9f2-328d01909222"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Flow_SignoffStatus xmlns="086b6104-a044-4b77-af40-37bf74d909c3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="223469b0-54b4-4219-b9f2-328d01909222" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="086b6104-a044-4b77-af40-37bf74d909c3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14E8A09A-F324-4A85-9420-4F283762450F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -1849,7 +2386,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{309E20D2-7E5E-4AEE-970F-82BFABC7C31E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1867,4 +2404,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6E18965-B26D-4362-B735-99223F49F9C5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="086b6104-a044-4b77-af40-37bf74d909c3"/>
+    <ds:schemaRef ds:uri="223469b0-54b4-4219-b9f2-328d01909222"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>